<commit_message>
Normaliza export CSV e atualiza manifesto de integridade
</commit_message>
<xml_diff>
--- a/public/levantamentos/politicas-ia/base-politicas-ia-2026-10-en.xlsx
+++ b/public/levantamentos/politicas-ia/base-politicas-ia-2026-10-en.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dataset" sheetId="1" r:id="Rd2b7cb1edfa34ba5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="2" r:id="R3b788e5595cf45cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dataset" sheetId="1" r:id="Ra832b3e07d28488b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="2" r:id="Rcad39a3f18d746c2"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Corrige significado geografico de AL no vocabulario e codebook ingles
</commit_message>
<xml_diff>
--- a/public/levantamentos/politicas-ia/base-politicas-ia-2026-10-en.xlsx
+++ b/public/levantamentos/politicas-ia/base-politicas-ia-2026-10-en.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dataset" sheetId="1" r:id="Ra832b3e07d28488b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="2" r:id="Rcad39a3f18d746c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dataset" sheetId="1" r:id="Rd27dece692a24981"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="2" r:id="R5327cd799fa24301"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -7013,7 +7013,7 @@
         <x:v>Geographical scope</x:v>
       </x:c>
       <x:c r="B11" s="8" t="str">
-        <x:v>Alemanha = Germany; Brasil = Brazil; Brasil/AL = Brazil/Alagoas; China = China; EUA = United States; Europa = Europe; Internacional = International; Reino Unido = United Kingdom; Suíça = Switzerland.</x:v>
+        <x:v>Alemanha = Germany; Brasil = Brazil; Brasil/AL = Brazil/Latin America; China = China; EUA = United States; Europa = Europe; Internacional = International; Reino Unido = United Kingdom; Suíça = Switzerland.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="39.599998474121094" hidden="0" customHeight="1">

</xml_diff>

<commit_message>
Atualiza auditoria semanal de políticas e exports PT/EN em 24/10
</commit_message>
<xml_diff>
--- a/public/levantamentos/politicas-ia/base-politicas-ia-2026-10-en.xlsx
+++ b/public/levantamentos/politicas-ia/base-politicas-ia-2026-10-en.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dataset" sheetId="1" r:id="Rd27dece692a24981"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="2" r:id="R5327cd799fa24301"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dataset" sheetId="1" r:id="Rd3e09aeb76d34be0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="2" r:id="Rea9e4dfaed514436"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3968,7 +3968,7 @@
       </x:c>
       <x:c r="O83" s="8"/>
     </x:row>
-    <x:row r="84" ht="66" hidden="0" customHeight="1">
+    <x:row r="84" ht="132" hidden="0" customHeight="1">
       <x:c r="A84" s="7" t="str">
         <x:v>Scientia Agricola (USP/ESALQ)</x:v>
       </x:c>
@@ -4004,7 +4004,7 @@
         <x:v>https://www.scielo.br/journal/sa/about/#instructions</x:v>
       </x:c>
       <x:c r="M84" s="8" t="str">
-        <x:v>Disclose tool, version, model and source in Materials and Methods when used for writing, images/graphics or data, plus a declaration before references. AI-translated texts are prohibited. The passage consulted does not require a non-use declaration and does not specifically regulate reviewers.</x:v>
+        <x:v>Disclose the tool, version, model and source in Materials and Methods when used for writing, images/graphics or data, as well as in a statement before References. Article Submission Format requires a Declaration of use of AI Technologies even when AI was not used; the previous description omitted this requirement. AI-translated texts are prohibited. Image use does not authorise fraudulent manipulation or data fabrication. The examined instructions contain no specific AI rule for reviewers. The date of the policy change is not stated; this descriptive correction was observed on 24 October 2026.</x:v>
       </x:c>
       <x:c r="N84" s="8" t="str">
         <x:v>Agricultural Sciences</x:v>
@@ -5149,7 +5149,7 @@
       </x:c>
       <x:c r="O110" s="8"/>
     </x:row>
-    <x:row r="111" ht="132" hidden="0" customHeight="1">
+    <x:row r="111" ht="158.39999389648438" hidden="0" customHeight="1">
       <x:c r="A111" s="7" t="str">
         <x:v>University of Chicago Press (livros)</x:v>
       </x:c>
@@ -5172,10 +5172,10 @@
         <x:v>Vedada</x:v>
       </x:c>
       <x:c r="H111" s="7" t="str">
-        <x:v>Múltiplos</x:v>
+        <x:v>Submissão/carta</x:v>
       </x:c>
       <x:c r="I111" s="7" t="str">
-        <x:v>Vedado</x:v>
+        <x:v>Condicionado</x:v>
       </x:c>
       <x:c r="J111" s="7" t="str">
         <x:v>Restritas</x:v>
@@ -5187,7 +5187,7 @@
         <x:v>https://press.uchicago.edu/resource/ai_guidelines.html</x:v>
       </x:c>
       <x:c r="M111" s="8" t="str">
-        <x:v>Books rule updated on 22 June 2026; journals have their own rules. Prohibits using AI to write/rewrite text or generate arguments; auxiliary research and superficial grammar correction are allowed. Report all use to the editor at submission and to readers in the book, normally in Acknowledgements and/or notes. Prohibits fabricating/altering illustrations, including redrawing maps, enlarging image files or adding/removing elements; visualising one's own data is allowed with disclosure. Requires unassisted reviews and prohibits uploading manuscripts, proposals or one's own review to AI, even if the tool promises not to retain data.</x:v>
+        <x:v>Book policy revised on 21 October 2026; journals have their own rules. AI may not write/rewrite text or generate arguments; auxiliary research and surface-level grammar corrections are allowed. All use must be disclosed to the acquisitions editor at submission; possible disclosure to readers is discussed with that editor, without a universally mandatory section. Fabricating or altering illustrations and maps, upscaling images, or adding/removing elements is prohibited; visualising the author’s own data is allowed with disclosure. Reviewers may consult AI as an online research tool, but may not summarise the work, develop arguments or write/rewrite their assessment; they may not upload any part of manuscripts or proposals to any AI tool.</x:v>
       </x:c>
       <x:c r="N111" s="8" t="str">
         <x:v>Humanities</x:v>
@@ -5239,7 +5239,7 @@
       </x:c>
       <x:c r="O112" s="8"/>
     </x:row>
-    <x:row r="113" ht="15" hidden="0" customHeight="1">
+    <x:row r="113" ht="171.60000610351562" hidden="0" customHeight="1">
       <x:c r="A113" s="7" t="str">
         <x:v>Rev. Brasileira de Ciências Sociais (ANPOCS)</x:v>
       </x:c>
@@ -5257,16 +5257,16 @@
       </x:c>
       <x:c r="F113" s="9"/>
       <x:c r="G113" s="7" t="str">
-        <x:v>Vedada</x:v>
+        <x:v>Permitida</x:v>
       </x:c>
       <x:c r="H113" s="7" t="str">
-        <x:v>—</x:v>
+        <x:v>Múltiplos</x:v>
       </x:c>
       <x:c r="I113" s="7" t="str">
-        <x:v>Não trata</x:v>
+        <x:v>Condicionado</x:v>
       </x:c>
       <x:c r="J113" s="7" t="str">
-        <x:v>Não trata</x:v>
+        <x:v>Restritas</x:v>
       </x:c>
       <x:c r="K113" s="7" t="str">
         <x:v>P</x:v>
@@ -5275,7 +5275,7 @@
         <x:v>https://www.scielo.br/journal/rbcsoc/about/#instructions</x:v>
       </x:c>
       <x:c r="M113" s="8" t="str">
-        <x:v>Does not accept chatbots or AI in producing texts.</x:v>
+        <x:v>The current policy allows generative-AI-assisted content under human responsibility, without assigning authorship to the tool. Information, references, plagiarism and rights must be checked. Disclose use in the cover letter and at the end of the manuscript, before References, specifying tool, model/version, date, purpose and human review. AI-generated images or audiovisual material are not accepted, except in articles specifically discussing these issues. Reviewers are strongly advised not to upload manuscripts or data to AI tools because of confidentiality; this recommendation does not authorise delegating assessment. Official Portuguese and English versions were checked; the date of change is not stated. The previous blanket-prohibition coding was corrected on 24 October 2026.</x:v>
       </x:c>
       <x:c r="N113" s="8" t="str">
         <x:v>Humanities</x:v>
@@ -5722,7 +5722,7 @@
         <x:v>Text generation: Sem regra → Permitida; Disclosure location: — → Múltiplos; Verification: A → P</x:v>
       </x:c>
     </x:row>
-    <x:row r="124" ht="105.5999984741211" hidden="0" customHeight="1">
+    <x:row r="124" ht="158.39999389648438" hidden="0" customHeight="1">
       <x:c r="A124" s="7" t="str">
         <x:v>Elsevier</x:v>
       </x:c>
@@ -5738,7 +5738,9 @@
       <x:c r="E124" s="7" t="str">
         <x:v>Internacional</x:v>
       </x:c>
-      <x:c r="F124" s="9"/>
+      <x:c r="F124" s="9" t="n">
+        <x:v>2026</x:v>
+      </x:c>
       <x:c r="G124" s="7" t="str">
         <x:v>Permitida</x:v>
       </x:c>
@@ -5758,7 +5760,7 @@
         <x:v>https://www.elsevier.com/about/policies-and-standards/generative-ai-policies-for-journals</x:v>
       </x:c>
       <x:c r="M124" s="8" t="str">
-        <x:v>Manuscript preparation: dedicated declaration; AI as a method: detailed Methods description. Basic corrections and accessibility have exemptions. Allows explanatory images disclosed in captions and the general declaration, and reproducible data-derived visualisations; prohibits fabricating primary data/images and using general GenAI in graphical abstracts. Reviewers may use only human-controlled assistance and private tools, with confidentiality and disclosure except for basic checks.</x:v>
+        <x:v>General policy updated in June 2026. Manuscript preparation: dedicated disclosure statement; AI as a method: detailed description in Methods. Basic checks and accessibility uses have exemptions. Disclosed explanatory images and reproducible data-derived visualisations are allowed; fabrication of primary data/images and general-purpose GenAI for graphical abstracts are prohibited. Reviewers may use only human-controlled assistance and private tools, preserving confidentiality and disclosing use beyond basic checks; confidential content must not be uploaded to external services. Editors may use approved internal systems while retaining human decisions. Identifying the year on 24 October supplements metadata; it is not a policy change dated to this week.</x:v>
       </x:c>
       <x:c r="N124" s="8" t="str">
         <x:v>Multidisciplinary / cross-disciplinary</x:v>
@@ -6989,7 +6991,7 @@
         <x:v>Reference date</x:v>
       </x:c>
       <x:c r="B8" s="8" t="str">
-        <x:v>Historical baseline: 2026-10-16. Full review: 2026-10-17; 149/149 records reconciled, 129 corrected, 0 unresolved. A/NL are limited to the described corpora, not universal absence. Detailed audit history (Portuguese): https://lapig-ufg.github.io/observatorio-ia/levantamentos/politicas-ia/revisao-2026-10-17.json</x:v>
+        <x:v>Historical baseline: 2026-10-16. Full review: 2026-10-24; 149/149 records reconciled, 4 corrected, 0 unresolved. A/NL are limited to the described corpora, not universal absence. Detailed audit history (Portuguese): https://lapig-ufg.github.io/observatorio-ia/levantamentos/politicas-ia/revisao-2026-10-24.json</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="26.399999618530273" hidden="0" customHeight="1">

</xml_diff>

<commit_message>
Atualiza políticas PT/EN em 31/10 com cobertura parcial explícita
</commit_message>
<xml_diff>
--- a/public/levantamentos/politicas-ia/base-politicas-ia-2026-10-en.xlsx
+++ b/public/levantamentos/politicas-ia/base-politicas-ia-2026-10-en.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dataset" sheetId="1" r:id="Rd3e09aeb76d34be0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="2" r:id="Rea9e4dfaed514436"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dataset" sheetId="1" r:id="Rc9af3bc5ec494283"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="2" r:id="R2901934c375942a3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -538,7 +538,7 @@
         <x:v>Disclosure location: Não especifica → Submissão/carta; Reviewers: Não trata → Condicionado; Source: www.csescienceeditor.org → www.cse-scienceeditor.org</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="105.5999984741211" hidden="0" customHeight="1">
+    <x:row r="6" ht="118.80000305175781" hidden="0" customHeight="1">
       <x:c r="A6" s="7" t="str">
         <x:v>EASE</x:v>
       </x:c>
@@ -576,7 +576,7 @@
         <x:v>https://ease.org.uk/2024/09/recommendations-on-the-use-of-ai-in-scholarly-communication/</x:v>
       </x:c>
       <x:c r="M6" s="8" t="str">
-        <x:v>EASE recommendations (2024), not automatically binding rules for every journal. Recommends disclosing use in creation/editing, including responses to reviews; methods/data/code in Methods or an AI statement, with visualisations also identified in captions. Each journal should specify whether language editing is exempt. Reviewers should follow the local policy and disclose assistance in creating/editing their review; detectors should not be used as conclusive evidence.</x:v>
+        <x:v>EASE recommendations (2024), not automatically binding rules for every journal. Recommends disclosing creation/editing uses, including responses to reviewers; methods/data/code in Methods or an AI statement, and visualisations also in captions. Each journal should specify whether language editing is exempt. Reviewers follow local policy and disclose assistance in creating/editing their report. For suspected breaches, recommends informing the editor and accepts detector reports as possible evidence; it does not define a threshold for conclusive proof.</x:v>
       </x:c>
       <x:c r="N6" s="8" t="str">
         <x:v>Multidisciplinary / cross-disciplinary</x:v>
@@ -718,7 +718,7 @@
       </x:c>
       <x:c r="O9" s="8"/>
     </x:row>
-    <x:row r="10" ht="132" hidden="0" customHeight="1">
+    <x:row r="10" ht="211.1999969482422" hidden="0" customHeight="1">
       <x:c r="A10" s="7" t="str">
         <x:v>ISTIC + editoras globais (China)</x:v>
       </x:c>
@@ -734,7 +734,9 @@
       <x:c r="E10" s="7" t="str">
         <x:v>China</x:v>
       </x:c>
-      <x:c r="F10" s="9"/>
+      <x:c r="F10" s="9" t="n">
+        <x:v>2025</x:v>
+      </x:c>
       <x:c r="G10" s="7" t="str">
         <x:v>Restrita</x:v>
       </x:c>
@@ -751,10 +753,10 @@
         <x:v>P</x:v>
       </x:c>
       <x:c r="L10" s="7" t="str">
-        <x:v>https://www.lib.szu.edu.cn/sites/szulib/files/2025-06/%E5%AD%A6%E6%9C%AF%E5%87%BA%E7%89%88%E4%B8%ADAIGC%E4%BD%BF%E7%94%A8%E8%BE%B9%E7%95%8C%E6%8C%87%E5%8D%972.0.pdf</x:v>
+        <x:v>https://rdswxb.hainanu.edu.cn/fileRDSWXB/cms/news/info/2026/01/c391fa83b285429f863b5dfc867936e0/%E5%AD%A6%E6%9C%AF%E5%87%BA%E7%89%88%E4%B8%ADAIGC%E4%BD%BF%E7%94%A8%E8%BE%B9%E7%95%8C%E6%8C%87%E5%8D%973.0%EF%BC%88%E4%B8%AD%E6%96%87%E7%89%88%EF%BC%89.pdf</x:v>
       </x:c>
       <x:c r="M10" s="8" t="str">
-        <x:v>AIGC Guide 2.0 developed by ISTIC with publishing partners; it does not replace each publisher's/journal's own policy. Allows assistance in writing and presenting real data under human responsibility and requests the tool, version, uses and affected parts in Methods or Acknowledgements. Reviewers may use only assistance allowed by the journal, without uploading confidential manuscripts. Fabricating experimental images and using AI in graphical abstracts are prohibited; cover art requires prior permission and appropriate rights. The normative year is not stated in the document consulted.</x:v>
+        <x:v>AIGC 3.0 guide from ISTIC and six publishers, released on 7 December 2025 according to the institute's official announcement; primary text checked in an institutional copy at Hainan University. Does not replace individual policies. Allows assistance with language, literature review and presentation of real data, without writing the entire paper or replacing human interpretation and conclusions. Disclose tool/version, dates, prompts, parts and records in Methods, notes, Acknowledgements or appendices. Reviewers follow the journal: assistance only with their own comments, without processing the manuscript; never send confidential content to public AI without authorisation. Authors must also not send identifiable reviews to public AI. Fabricated experimental images and AI in graphical abstracts are prohibited; covers require permission and rights. The 2.0 reference was replaced on 31 October 2026, without claiming a release during this week.</x:v>
       </x:c>
       <x:c r="N10" s="8" t="str">
         <x:v>Multidisciplinary / cross-disciplinary</x:v>
@@ -1225,10 +1227,10 @@
         <x:v>2026</x:v>
       </x:c>
       <x:c r="G21" s="7" t="str">
-        <x:v>N/A</x:v>
+        <x:v>Permitida</x:v>
       </x:c>
       <x:c r="H21" s="7" t="str">
-        <x:v>—</x:v>
+        <x:v>Sem exigência p/ redação</x:v>
       </x:c>
       <x:c r="I21" s="7" t="str">
         <x:v>Condicionado</x:v>
@@ -1561,7 +1563,7 @@
       </x:c>
       <x:c r="O28" s="8"/>
     </x:row>
-    <x:row r="29" ht="79.19999694824219" hidden="0" customHeight="1">
+    <x:row r="29" ht="105.5999984741211" hidden="0" customHeight="1">
       <x:c r="A29" s="7" t="str">
         <x:v>USGS</x:v>
       </x:c>
@@ -1582,7 +1584,7 @@
         <x:v>Permitida</x:v>
       </x:c>
       <x:c r="H29" s="7" t="str">
-        <x:v>Não especifica</x:v>
+        <x:v>Múltiplos</x:v>
       </x:c>
       <x:c r="I29" s="7" t="str">
         <x:v>Não trata</x:v>
@@ -1597,7 +1599,7 @@
         <x:v>https://www.usgs.gov/office-of-science-quality-and-integrity/example-ai-disclosure-statements-usgs-scientific</x:v>
       </x:c>
       <x:c r="M29" s="8" t="str">
-        <x:v>Guidance for USGS scientific products, not a general funding rule. Generative AI, including images, requires transparency and human verification. The page provides disclosure templates without prescribing a section. Specific machine learning may not require a separate disclosure when the method is already described/cited; the page does not regulate reviewers.</x:v>
+        <x:v>Guidance for USGS scientific products, not a general funding rule. Generative AI, including images, requires transparency and human verification. Disclose design, analysis and code in Methods; writing, editing, images and ideas in Acknowledgements; publishable details, such as tool, version, prompts and dates, in supplements. Specific machine learning may not require a separate declaration when techniques are described/cited according to USGS practice. AI cannot be an author; this page does not establish a reviewer rule.</x:v>
       </x:c>
       <x:c r="N29" s="8" t="str">
         <x:v>Exact and Earth Sciences</x:v>
@@ -1690,7 +1692,7 @@
       </x:c>
       <x:c r="O31" s="8"/>
     </x:row>
-    <x:row r="32" ht="15" hidden="0" customHeight="1">
+    <x:row r="32" ht="132" hidden="0" customHeight="1">
       <x:c r="A32" s="7" t="str">
         <x:v>Royal Society of Chemistry</x:v>
       </x:c>
@@ -1714,7 +1716,7 @@
         <x:v>Múltiplos</x:v>
       </x:c>
       <x:c r="I32" s="7" t="str">
-        <x:v>Não trata</x:v>
+        <x:v>Condicionado</x:v>
       </x:c>
       <x:c r="J32" s="7" t="str">
         <x:v>Restritas</x:v>
@@ -1726,7 +1728,7 @@
         <x:v>https://www.rsc.org/publishing/journals/processes-and-policies/author-responsibilities</x:v>
       </x:c>
       <x:c r="M32" s="8" t="str">
-        <x:v>Cover letter plus Experimental plus Acknowledgements.</x:v>
+        <x:v>Disclose AI use in the cover letter, in Experimental/Methods with prompts, and in Acknowledgements with the tool/version; simple assistive editing is exempt. Humans remain fully responsible. Aesthetic illustrations require licensed training data, commercial rights and a caption; identifiable people and manipulation of data features are not accepted, except as a reproducible research method. Reviewers may only improve the language of their own report in a system without retention/training, with disclosure in confidential comments to the editor; they must not generate an assessment or upload manuscripts or supplements.</x:v>
       </x:c>
       <x:c r="N32" s="8" t="str">
         <x:v>Exact and Earth Sciences</x:v>
@@ -1864,7 +1866,7 @@
       </x:c>
       <x:c r="O35" s="8"/>
     </x:row>
-    <x:row r="36" ht="184.8000030517578" hidden="0" customHeight="1">
+    <x:row r="36" ht="171.60000610351562" hidden="0" customHeight="1">
       <x:c r="A36" s="7" t="str">
         <x:v>IJRS / GIScience &amp; RS / Remote Sensing Letters</x:v>
       </x:c>
@@ -1900,7 +1902,7 @@
         <x:v>https://taylorandfrancis.com/our-policies/ai-policy/</x:v>
       </x:c>
       <x:c r="M36" s="8" t="str">
-        <x:v>IJRS (guide updated 29 September 2025), GIScience &amp; Remote Sensing (12 October 2026) and Remote Sensing Letters (14 September 2026) require a statement of AI use or non-use in research and manuscript preparation and refer to T&amp;F rules. State the tool, version, purpose and manner of use; the guides prescribe no single section. The general policy requires rigorous human review and prohibits replacing intellectual responsibilities. Disclosed visualisations and conceptual illustrations are allowed, not fabrication/manipulation of results, samples or diagnostic images. Reviewers may only improve the language of their own review, without manuscript uploads, automated analysis/summary or generation of an assessment. All three guides were consulted separately; inheritance does not follow merely from the commercial relationship.</x:v>
+        <x:v>IJRS (guide updated 29 September 2025), GIScience &amp; Remote Sensing (12 October 2026) and Remote Sensing Letters (20 October 2026) require a declaration of AI use or non-use in research and manuscript preparation and refer to T&amp;F rules. State the tool, version, purpose and manner of use; the guides do not prescribe a single section. The general policy requires rigorous human review and prohibits replacing intellectual responsibilities. Disclosed visualisations and conceptual illustrations are allowed, not fabrication/manipulation of results, specimens or diagnostic images. Reviewers may only improve the language of their own report, without uploading manuscripts, automated analysis/summarisation or generating an assessment. Applicability was checked separately in all three guides.</x:v>
       </x:c>
       <x:c r="N36" s="8" t="str">
         <x:v>Exact and Earth Sciences</x:v>
@@ -1995,7 +1997,7 @@
       </x:c>
       <x:c r="O38" s="8"/>
     </x:row>
-    <x:row r="39" ht="118.80000305175781" hidden="0" customHeight="1">
+    <x:row r="39" ht="132" hidden="0" customHeight="1">
       <x:c r="A39" s="7" t="str">
         <x:v>Boletim de Ciências Geodésicas</x:v>
       </x:c>
@@ -2031,14 +2033,14 @@
         <x:v>https://www.scielo.br/journal/bcg/about/?ilang=en</x:v>
       </x:c>
       <x:c r="M39" s="8" t="str">
-        <x:v>No specific AI clause on writing, disclosure, reviews or illustrations was found in the full instructions available on SciELO. The journal refers to FAPESP's 2014 Code of Good Scientific Practice, which establishes responsibility, authorship, data integrity and confidentiality, without a specific generative-AI regime in the sections examined. The UFPR submission portal was under maintenance. The coded absence is limited to this accessible normative corpus; it certifies neither the absence of additional instructions nor permission to use AI.</x:v>
+        <x:v>The public instructions examined on SciELO and the UFPR portal regulate originality, data integrity, human authorship, confidentiality and assessment. The journal's own portal is accessible and states that it does not accept submissions there; the SciELO page directs submissions to ScholarOne. BCG explicitly refers to FAPESP's 2014 code, with no specific GenAI clause in the examined authorship, data and reviewing sections. No explicit AI rule in this corpus; this establishes neither permission nor universal absence. Later agency guidance was not inherited without demonstrated adoption.</x:v>
       </x:c>
       <x:c r="N39" s="8" t="str">
         <x:v>Exact and Earth Sciences</x:v>
       </x:c>
       <x:c r="O39" s="8"/>
     </x:row>
-    <x:row r="40" ht="92.4000015258789" hidden="0" customHeight="1">
+    <x:row r="40" ht="118.80000305175781" hidden="0" customHeight="1">
       <x:c r="A40" s="7" t="str">
         <x:v>Química Nova (SBQ)</x:v>
       </x:c>
@@ -2059,7 +2061,7 @@
         <x:v>Permitida</x:v>
       </x:c>
       <x:c r="H40" s="7" t="str">
-        <x:v>Submissão/carta</x:v>
+        <x:v>Múltiplos</x:v>
       </x:c>
       <x:c r="I40" s="7" t="str">
         <x:v>Não trata</x:v>
@@ -2074,7 +2076,7 @@
         <x:v>https://www.scielo.br/journal/qn/about/</x:v>
       </x:c>
       <x:c r="M40" s="8" t="str">
-        <x:v>Responsible use is accepted with human oversight and scientific reasoning. Disclosure is mandatory in ScholarOne, stating the tool/model and purpose; manuscript disclosure is offered as a possibility, without a fixed section. The policy mentions figures/tables but establishes no independent visual rule. AI is not a co-author; references, data and results must be verified. This section has no specific AI rule for reviewers.</x:v>
+        <x:v>Responsible use is accepted under human supervision and scientific reasoning. Instruction 2.3 requires disclosing the stage/purpose in the manuscript and the tool/model in ScholarOne; it does not prescribe a single section. There is an internal difference: the general block describes manuscript disclosure as a possibility, while 2.3 requires it. Mention of figures/tables does not establish an independent image rule. AI is not a co-author; references, data and results must be verified without exposing confidential or personal data. The clause has no specific reviewer AI rule.</x:v>
       </x:c>
       <x:c r="N40" s="8" t="str">
         <x:v>Exact and Earth Sciences</x:v>
@@ -2119,7 +2121,7 @@
         <x:v>https://proceedings.science/cfp/sbsr-2027?lang=pt-br</x:v>
       </x:c>
       <x:c r="M41" s="8" t="str">
-        <x:v>The paper rules for the XXII SBSR, the April 2027 edition already accepting submissions in 2026, contain no specific AI clause on writing, disclosure, reviews or images. They require originality, rigorous data, correct authorship and assessment by an independent committee. The absence is limited to these PT/EN rules; it is neither implicit permission nor an INPE institutional AI policy. The versions differ on the submission deadline, and the English version retains a reference to edition XXI; the Portuguese page identifies the current edition and extension. The edition year was not treated as the rule's publication date.</x:v>
+        <x:v>The paper rules for the XXII SBSR, the April 2027 edition open for submissions in 2026, contain no specific AI clause for writing, disclosure, reviewing or images. They require originality, rigorous data, correct authorship and assessment by an independent committee. Absence is bounded to these Portuguese/English pages; it establishes neither implicit permission nor an INPE institutional AI policy. At the current consultation, both state 6 November 2026 as the deadline; the English page still contains a residual reference to edition XXI. The event year was not treated as the rule's publication date.</x:v>
       </x:c>
       <x:c r="N41" s="8" t="str">
         <x:v>Exact and Earth Sciences</x:v>
@@ -2341,7 +2343,7 @@
       </x:c>
       <x:c r="O46" s="8"/>
     </x:row>
-    <x:row r="47" ht="145.1999969482422" hidden="0" customHeight="1">
+    <x:row r="47" ht="158.39999389648438" hidden="0" customHeight="1">
       <x:c r="A47" s="7" t="str">
         <x:v>Society for Neuroscience (J. Neurosci.)</x:v>
       </x:c>
@@ -2379,7 +2381,7 @@
         <x:v>https://www.jneurosci.org/content/information-authors</x:v>
       </x:c>
       <x:c r="M47" s="8" t="str">
-        <x:v>The September 2026 instructions allow AI language editing and require disclosure in Acknowledgements at submission. This editing permission was not extended to autonomous scientific-content generation. SfN rules, expressly adopted by the journal, prohibit sharing manuscripts or confidential information with AI. Conditional codes this upload prohibition: the rule neither expressly authorises review editing there nor literally prohibits all auxiliary uses. Image features must not be selectively introduced, obscured, moved or removed; adjustments must be uniform and transparent, preserving the original. These visual-integrity requirements are not blanket permission for synthetic illustrations.</x:v>
+        <x:v>The October 2026 instructions allow AI for language editing and require disclosure in Acknowledgements at submission. This editing permission was not extended to autonomous generation of scientific content. SfN rules, explicitly adopted by the journal, prohibit sharing manuscripts or confidential information with AI. Conditional codes this upload prohibition: that provision neither expressly authorises editing reports nor literally prohibits all auxiliary uses. Images must not have features selectively introduced, obscured, moved or removed; adjustments must be uniform and transparent, with originals retained. These visual-integrity requirements do not constitute general permission for synthetic illustrations.</x:v>
       </x:c>
       <x:c r="N47" s="8" t="str">
         <x:v>Biological Sciences</x:v>
@@ -2515,7 +2517,7 @@
       </x:c>
       <x:c r="O50" s="8"/>
     </x:row>
-    <x:row r="51" ht="66" hidden="0" customHeight="1">
+    <x:row r="51" ht="132" hidden="0" customHeight="1">
       <x:c r="A51" s="7" t="str">
         <x:v>Genetics and Molecular Biology (SBG)</x:v>
       </x:c>
@@ -2551,7 +2553,7 @@
         <x:v>https://www.scielo.br/journal/gmb/about/?ilang=en</x:v>
       </x:c>
       <x:c r="M51" s="8" t="str">
-        <x:v>Disclose use in the cover letter and Statements section; document LLM use in Methods or an appropriate part. Assistive copyediting of human text is exempt, not autonomous generation. The section consulted establishes neither specific image permission nor a reviewer rule.</x:v>
+        <x:v>Disclose use in the cover letter and Statements; document LLM use in Methods or an appropriate section. The general section exempts assistive copyediting of human-written text, but the Artificial Intelligence Statement requests disclosure of generation in writing/figures or use solely to correct English. The instructions contain this internal difference; an unconditional disclosure exemption should not be assumed. Authorship and responsibility remain human. Mention of figures does not prescribe an independent image regime; the examined sections have no specific reviewer GenAI rule.</x:v>
       </x:c>
       <x:c r="N51" s="8" t="str">
         <x:v>Biological Sciences</x:v>
@@ -2945,7 +2947,7 @@
         <x:v>A</x:v>
       </x:c>
       <x:c r="L60" s="7" t="str">
-        <x:v>https://www.abes-dn.org.br/wp-content/uploads/2025/09/Guidelines-ESA-Journal_Aug_25.pdf</x:v>
+        <x:v>https://abes-dn.org.br/wp-content/uploads/2025/09/Guidelines-ESA-Journal_Aug_25.pdf</x:v>
       </x:c>
       <x:c r="M60" s="8" t="str">
         <x:v>The full official August 2025 regulations, linked by ABES, contain no specific AI clause on writing, disclosure, reviews or images. They require originality, reproducible methods, references, mandatory figure provenance and author responsibility, and provide for human assessment by reviewers and editors. The coded absence is limited to these regulations and the SciELO instructions examined; it implies neither AI permission nor the absence of other editorial guidance.</x:v>
@@ -2955,7 +2957,7 @@
       </x:c>
       <x:c r="O60" s="8"/>
     </x:row>
-    <x:row r="61" ht="79.19999694824219" hidden="0" customHeight="1">
+    <x:row r="61" ht="105.5999984741211" hidden="0" customHeight="1">
       <x:c r="A61" s="7" t="str">
         <x:v>Rev. Brasileira de Recursos Hídricos (ABRHidro)</x:v>
       </x:c>
@@ -2991,7 +2993,7 @@
         <x:v>https://www.scielo.br/journal/rbrh/about/</x:v>
       </x:c>
       <x:c r="M61" s="8" t="str">
-        <x:v>Use in generation, analysis or revision must be disclosed in Materials and Methods, with extent, tool and parameters. Recommends the SciELO guide to authors and reviewers, without its own specific reviewer/image rule in the clause. The source contains an incongruous reference to RDBCI, recorded as an editorial limitation.</x:v>
+        <x:v>Use for generation, analysis, revision or any other purpose must be disclosed in Materials and Methods, with extent, tool, version/model, source and parameters. Human authors remain responsible for originality, accuracy and limitations. Recommends the SciELO guide to authors and reviewers, without its own specific reviewer or image rule in that block. At the 31 October 2026 consultation, the journal identification in the passage is RBRH; the previous inconsistent mention of RDBCI no longer appears.</x:v>
       </x:c>
       <x:c r="N61" s="8" t="str">
         <x:v>Engineering</x:v>
@@ -4142,7 +4144,7 @@
         <x:v>Text generation: Sem regra → Permitida; Disclosure location: — → Não especifica; Verification: A → P</x:v>
       </x:c>
     </x:row>
-    <x:row r="88" ht="105.5999984741211" hidden="0" customHeight="1">
+    <x:row r="88" ht="118.80000305175781" hidden="0" customHeight="1">
       <x:c r="A88" s="7" t="str">
         <x:v>Ciência Rural (UFSM)</x:v>
       </x:c>
@@ -4178,7 +4180,7 @@
         <x:v>https://www.scielo.br/journal/cr/about/</x:v>
       </x:c>
       <x:c r="M88" s="8" t="str">
-        <x:v>Does not allow AI to write the manuscript, abstract, keywords, hypotheses or conclusion. Allows language revision and image improvement without adding/removing elements that change interpretation, under supervision and with disclosure in an appropriate section. AI integrated into methodology must be described reproducibly in Materials and Methods. The page prescribes neither a single declaration heading nor its own reviewer rule.</x:v>
+        <x:v>Does not allow AI to write the manuscript, abstract, keywords, hypotheses or conclusion. Allows language revision and image improvement without adding/removing elements that change interpretation, under supervision and with disclosure. The general block asks for an appropriate section; the article structure also includes a Declaration of Use of Artificial Intelligence before References. AI integrated into the methodology must be described reproducibly in Materials and Methods. The examined sections have no specific reviewer GenAI rule.</x:v>
       </x:c>
       <x:c r="N88" s="8" t="str">
         <x:v>Agricultural Sciences</x:v>
@@ -4614,7 +4616,7 @@
         <x:v>https://www.e-elgar.com/author-hub/as-you-write-your-book-or-chapter/</x:v>
       </x:c>
       <x:c r="M98" s="8" t="str">
-        <x:v>Rule for books/chapters: does not allow writing, rewriting or paraphrasing with GenAI; limited language checkers are allowed. Use beyond minor assistance must be disclosed in the proposal, checklist and manuscript when required. Do not include generated images without prior discussion with the editor; fabricating/manipulating original data or images is prohibited. The page establishes no specific AI reviewer rule. No explicit normative date.</x:v>
+        <x:v>Rule for books/chapters: GenAI must not write, rewrite or paraphrase text; limited language checkers are allowed. Use beyond minor support must be disclosed in the proposal, checklist and manuscript where required, with tool/version/provider and purpose. Fabricating, altering or manipulating original research data, results or images, or violating confidentiality or rights, is prohibited. The examined page establishes neither a specific reviewer AI rule nor an explicit policy date.</x:v>
       </x:c>
       <x:c r="N98" s="8" t="str">
         <x:v>Applied Social Sciences</x:v>
@@ -6332,7 +6334,7 @@
       </x:c>
       <x:c r="O137" s="8"/>
     </x:row>
-    <x:row r="138" ht="79.19999694824219" hidden="0" customHeight="1">
+    <x:row r="138" ht="145.1999969482422" hidden="0" customHeight="1">
       <x:c r="A138" s="7" t="str">
         <x:v>Royal Society (periódicos)</x:v>
       </x:c>
@@ -6356,7 +6358,7 @@
         <x:v>Não especifica</x:v>
       </x:c>
       <x:c r="I138" s="7" t="str">
-        <x:v>Não trata</x:v>
+        <x:v>Condicionado</x:v>
       </x:c>
       <x:c r="J138" s="7" t="str">
         <x:v>Não trata</x:v>
@@ -6368,7 +6370,7 @@
         <x:v>https://royalsociety.org/journals/ethics-policies/artificial-intelligence/</x:v>
       </x:c>
       <x:c r="M138" s="8" t="str">
-        <x:v>For writing, AI only for language and readability, with disclosure including language editing. It must not replace insights, analysis/interpretation or conclusions. Code/method searches and protein-structure prediction are allowed. The declaration must appear in the manuscript and published work, without a fixed section; this page establishes no specific reviewer or image rule.</x:v>
+        <x:v>For writing, AI is limited to language and readability, with disclosure including language editing. It does not replace insights, analysis/interpretation or conclusions. Code/method searches and protein-structure prediction are allowed. Disclose in the manuscript and published work, without a prescribed section. The editorial standards policy prohibits reviewers from entering manuscript details into generative AI tools because of confidentiality; it does not establish a prohibition on every assistive task. The AI page has no separate regime for generated images. Adding the reviewer clause corrects the description's coverage without establishing when the rule changed.</x:v>
       </x:c>
       <x:c r="N138" s="8" t="str">
         <x:v>Multidisciplinary / cross-disciplinary</x:v>
@@ -6692,7 +6694,7 @@
       </x:c>
       <x:c r="O145" s="8"/>
     </x:row>
-    <x:row r="146" ht="15" hidden="0" customHeight="1">
+    <x:row r="146" ht="132" hidden="0" customHeight="1">
       <x:c r="A146" s="7" t="str">
         <x:v>ERC</x:v>
       </x:c>
@@ -6730,7 +6732,7 @@
         <x:v>https://erc.europa.eu/news-events/news/erc-clarifies-limits-ai-use-grant-evaluation</x:v>
       </x:c>
       <x:c r="M146" s="8" t="str">
-        <x:v>Assessors must not summarise, assess or draft with AI.</x:v>
+        <x:v>ERC guidance of 23 March 2026 for proposal assessment: AI does not replace full reading, summarisation, scientific judgement or the first draft of a review. It may correct language or translate the reviewer's own text and, in a secure local environment, expand their own notes into paragraphs without new arguments, interpretations or assessments; original wording is preferred. Never send proposals or confidential information to external services. Institutional systems require safeguards against retention, training or unauthorised access and do not remove human responsibility. This record concerns assessment, not authors writing journal articles.</x:v>
       </x:c>
       <x:c r="N146" s="8" t="str">
         <x:v>Multidisciplinary / cross-disciplinary</x:v>
@@ -6991,7 +6993,7 @@
         <x:v>Reference date</x:v>
       </x:c>
       <x:c r="B8" s="8" t="str">
-        <x:v>Historical baseline: 2026-10-16. Full review: 2026-10-24; 149/149 records reconciled, 4 corrected, 0 unresolved. A/NL are limited to the described corpora, not universal absence. Detailed audit history (Portuguese): https://lapig-ufg.github.io/observatorio-ia/levantamentos/politicas-ia/revisao-2026-10-24.json</x:v>
+        <x:v>Historical baseline: 2026-10-16. Last full reference: 2026-10-24. Partial review: 2026-10-31; 148/149 records reconciled, 17 corrected, 1 unresolved. A/NL are limited to the described corpora, not universal absence. Detailed audit history (Portuguese): https://lapig-ufg.github.io/observatorio-ia/levantamentos/politicas-ia/revisao-2026-10-31.json</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="26.399999618530273" hidden="0" customHeight="1">

</xml_diff>